<commit_message>
Rasy.xlsx: dodaj Jagdterrier (R331), mapa końcowa z decyzjami, reguły dopasowania nazw w DECYZJE.md
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Q2pg3BaaiyphGsjSqASTzq
</commit_message>
<xml_diff>
--- a/data/Rasy.xlsx
+++ b/data/Rasy.xlsx
@@ -170,7 +170,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Tabela1" displayName="Tabela1" ref="A1:AB331" headerRowCount="1" totalsRowShown="0" headerRowDxfId="0">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Tabela1" displayName="Tabela1" ref="A1:AB332" headerRowCount="1" totalsRowShown="0" headerRowDxfId="0">
   <autoFilter ref="A1:AB331"/>
   <sortState ref="A8:AB330">
     <sortCondition ref="C1:C331"/>
@@ -602,7 +602,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AB331"/>
+  <dimension ref="A1:AB332"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="2"/>
@@ -37263,6 +37263,127 @@
       <c r="Z331" t="inlineStr">
         <is>
           <t>zatwierdzone (właścicielka)</t>
+        </is>
+      </c>
+    </row>
+    <row r="332">
+      <c r="A332" t="inlineStr">
+        <is>
+          <t>R331</t>
+        </is>
+      </c>
+      <c r="B332" t="inlineStr">
+        <is>
+          <t>pies</t>
+        </is>
+      </c>
+      <c r="C332" t="inlineStr">
+        <is>
+          <t>Jagdterrier</t>
+        </is>
+      </c>
+      <c r="F332" t="n">
+        <v>2</v>
+      </c>
+      <c r="G332" t="n">
+        <v>0</v>
+      </c>
+      <c r="H332" t="n">
+        <v>0</v>
+      </c>
+      <c r="I332" t="inlineStr">
+        <is>
+          <t>Jagdterrier (2)</t>
+        </is>
+      </c>
+      <c r="J332" t="inlineStr">
+        <is>
+          <t>Jagdterrier</t>
+        </is>
+      </c>
+      <c r="K332" t="inlineStr">
+        <is>
+          <t>Niemiecki terier myśliwski</t>
+        </is>
+      </c>
+      <c r="L332" t="inlineStr">
+        <is>
+          <t>szkic (Claude, 2026-10-25)</t>
+        </is>
+      </c>
+      <c r="M332" t="inlineStr">
+        <is>
+          <t>Deutscher Jagdterrier</t>
+        </is>
+      </c>
+      <c r="N332" t="inlineStr">
+        <is>
+          <t>szkic (Claude, 2026-10-25)</t>
+        </is>
+      </c>
+      <c r="O332" t="inlineStr">
+        <is>
+          <t>Terrier de chasse allemand</t>
+        </is>
+      </c>
+      <c r="P332" t="inlineStr">
+        <is>
+          <t>szkic (Claude, 2026-10-25)</t>
+        </is>
+      </c>
+      <c r="Q332" t="inlineStr">
+        <is>
+          <t>Terrier de caza alemán</t>
+        </is>
+      </c>
+      <c r="R332" t="inlineStr">
+        <is>
+          <t>szkic (Claude, 2026-10-25)</t>
+        </is>
+      </c>
+      <c r="S332" t="inlineStr">
+        <is>
+          <t>Duitse jachtterriër</t>
+        </is>
+      </c>
+      <c r="T332" t="inlineStr">
+        <is>
+          <t>szkic (Claude, 2026-10-25)</t>
+        </is>
+      </c>
+      <c r="U332" t="inlineStr">
+        <is>
+          <t>Terrier da caccia tedesco</t>
+        </is>
+      </c>
+      <c r="V332" t="inlineStr">
+        <is>
+          <t>szkic (Claude, 2026-10-25)</t>
+        </is>
+      </c>
+      <c r="W332" t="inlineStr">
+        <is>
+          <t>Terrier de caça alemão</t>
+        </is>
+      </c>
+      <c r="X332" t="inlineStr">
+        <is>
+          <t>szkic (Claude, 2026-10-25)</t>
+        </is>
+      </c>
+      <c r="Y332" t="inlineStr">
+        <is>
+          <t>Tysk jaktterrier</t>
+        </is>
+      </c>
+      <c r="Z332" t="inlineStr">
+        <is>
+          <t>szkic (Claude, 2026-10-25)</t>
+        </is>
+      </c>
+      <c r="AB332" t="inlineStr">
+        <is>
+          <t>Dodana 25.10.2026 na polecenie właścicielki (oferta płytki Jagdterrier, folder 174). Wszystkie tłumaczenia to szkice Claude'a: PL sprawdza właścicielka, pozostałe języki osoba natywna.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Rasy.xlsx: zatwierdzone tłumaczenia Jagdterrier; wzorce tytułu i tagów płytki (wersja robocza)
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Q2pg3BaaiyphGsjSqASTzq
</commit_message>
<xml_diff>
--- a/data/Rasy.xlsx
+++ b/data/Rasy.xlsx
@@ -37308,7 +37308,7 @@
       </c>
       <c r="L332" t="inlineStr">
         <is>
-          <t>szkic (Claude, 2026-10-25)</t>
+          <t>zatwierdzone (właścicielka)</t>
         </is>
       </c>
       <c r="M332" t="inlineStr">
@@ -37318,7 +37318,7 @@
       </c>
       <c r="N332" t="inlineStr">
         <is>
-          <t>szkic (Claude, 2026-10-25)</t>
+          <t>zatwierdzone (właścicielka)</t>
         </is>
       </c>
       <c r="O332" t="inlineStr">
@@ -37328,7 +37328,7 @@
       </c>
       <c r="P332" t="inlineStr">
         <is>
-          <t>szkic (Claude, 2026-10-25)</t>
+          <t>zatwierdzone (właścicielka)</t>
         </is>
       </c>
       <c r="Q332" t="inlineStr">
@@ -37338,7 +37338,7 @@
       </c>
       <c r="R332" t="inlineStr">
         <is>
-          <t>szkic (Claude, 2026-10-25)</t>
+          <t>zatwierdzone (właścicielka)</t>
         </is>
       </c>
       <c r="S332" t="inlineStr">
@@ -37348,7 +37348,7 @@
       </c>
       <c r="T332" t="inlineStr">
         <is>
-          <t>szkic (Claude, 2026-10-25)</t>
+          <t>zatwierdzone (właścicielka)</t>
         </is>
       </c>
       <c r="U332" t="inlineStr">
@@ -37358,7 +37358,7 @@
       </c>
       <c r="V332" t="inlineStr">
         <is>
-          <t>szkic (Claude, 2026-10-25)</t>
+          <t>zatwierdzone (właścicielka)</t>
         </is>
       </c>
       <c r="W332" t="inlineStr">
@@ -37368,7 +37368,7 @@
       </c>
       <c r="X332" t="inlineStr">
         <is>
-          <t>szkic (Claude, 2026-10-25)</t>
+          <t>zatwierdzone (właścicielka)</t>
         </is>
       </c>
       <c r="Y332" t="inlineStr">
@@ -37378,12 +37378,12 @@
       </c>
       <c r="Z332" t="inlineStr">
         <is>
-          <t>szkic (Claude, 2026-10-25)</t>
+          <t>zatwierdzone (właścicielka)</t>
         </is>
       </c>
       <c r="AB332" t="inlineStr">
         <is>
-          <t>Dodana 25.10.2026 na polecenie właścicielki (oferta płytki Jagdterrier, folder 174). Wszystkie tłumaczenia to szkice Claude'a: PL sprawdza właścicielka, pozostałe języki osoba natywna.</t>
+          <t>Dodana 25.10.2026 na polecenie właścicielki (oferta płytki Jagdterrier, folder 174). Tłumaczenia we wszystkich 8 językach zatwierdziła właścicielka 25.10.2026 (to nie jest weryfikacja natywna).</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Rasy.xlsx: R332 English Pointer, R333 German Longhaired Pointer (szkice); rozstrzygnięcia właścicielki; słowa odmian; partia 6 w toku
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_019xek4mwGKLwNoADM59d9Qh
</commit_message>
<xml_diff>
--- a/data/Rasy.xlsx
+++ b/data/Rasy.xlsx
@@ -602,7 +602,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AB332"/>
+  <dimension ref="A1:AB334"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="2"/>
@@ -4752,7 +4752,7 @@
       </c>
       <c r="AB36" t="inlineStr">
         <is>
-          <t>Do sprawdzenia, czy chodzi o English Pointer (nie pointera niemieckiego).</t>
+          <t>Do sprawdzenia, czy chodzi o English Pointer (nie pointera niemieckiego). Rozstrzygnięte 27.10.2026: oferta 664717946 to Pointer bez dopisków; English Pointer to osobny wiersz R332.</t>
         </is>
       </c>
     </row>
@@ -37384,6 +37384,238 @@
       <c r="AB332" t="inlineStr">
         <is>
           <t>Dodana 25.10.2026 na polecenie właścicielki (oferta płytki Jagdterrier, folder 174). Tłumaczenia we wszystkich 8 językach zatwierdziła właścicielka 25.10.2026 (to nie jest weryfikacja natywna).</t>
+        </is>
+      </c>
+    </row>
+    <row r="333">
+      <c r="A333" t="inlineStr">
+        <is>
+          <t>R332</t>
+        </is>
+      </c>
+      <c r="B333" t="inlineStr">
+        <is>
+          <t>pies</t>
+        </is>
+      </c>
+      <c r="C333" t="inlineStr">
+        <is>
+          <t>English Pointer</t>
+        </is>
+      </c>
+      <c r="F333" t="n">
+        <v>1</v>
+      </c>
+      <c r="G333" t="n">
+        <v>0</v>
+      </c>
+      <c r="H333" t="n">
+        <v>0</v>
+      </c>
+      <c r="I333" t="inlineStr">
+        <is>
+          <t>English Pointer (1)</t>
+        </is>
+      </c>
+      <c r="J333" t="inlineStr">
+        <is>
+          <t>Pointer angielski</t>
+        </is>
+      </c>
+      <c r="L333" t="inlineStr">
+        <is>
+          <t>szkic (Claude, 27.10.2026)</t>
+        </is>
+      </c>
+      <c r="M333" t="inlineStr">
+        <is>
+          <t>English Pointer</t>
+        </is>
+      </c>
+      <c r="N333" t="inlineStr">
+        <is>
+          <t>szkic (Claude, 27.10.2026)</t>
+        </is>
+      </c>
+      <c r="O333" t="inlineStr">
+        <is>
+          <t>Pointer anglais</t>
+        </is>
+      </c>
+      <c r="P333" t="inlineStr">
+        <is>
+          <t>szkic (Claude, 27.10.2026)</t>
+        </is>
+      </c>
+      <c r="Q333" t="inlineStr">
+        <is>
+          <t>Pointer inglés</t>
+        </is>
+      </c>
+      <c r="R333" t="inlineStr">
+        <is>
+          <t>szkic (Claude, 27.10.2026)</t>
+        </is>
+      </c>
+      <c r="S333" t="inlineStr">
+        <is>
+          <t>Engelse pointer</t>
+        </is>
+      </c>
+      <c r="T333" t="inlineStr">
+        <is>
+          <t>szkic (Claude, 27.10.2026)</t>
+        </is>
+      </c>
+      <c r="U333" t="inlineStr">
+        <is>
+          <t>Pointer inglese</t>
+        </is>
+      </c>
+      <c r="V333" t="inlineStr">
+        <is>
+          <t>szkic (Claude, 27.10.2026)</t>
+        </is>
+      </c>
+      <c r="W333" t="inlineStr">
+        <is>
+          <t>Pointer inglês</t>
+        </is>
+      </c>
+      <c r="X333" t="inlineStr">
+        <is>
+          <t>szkic (Claude, 27.10.2026)</t>
+        </is>
+      </c>
+      <c r="Y333" t="inlineStr">
+        <is>
+          <t>Engelsk pointer</t>
+        </is>
+      </c>
+      <c r="Z333" t="inlineStr">
+        <is>
+          <t>szkic (Claude, 27.10.2026)</t>
+        </is>
+      </c>
+      <c r="AB333" t="inlineStr">
+        <is>
+          <t>Dodana 27.10.2026 na polecenie właścicielki (rasa wskazana dla oferty 664703588). Tłumaczenia to szkice Claude'a do sprawdzenia.</t>
+        </is>
+      </c>
+    </row>
+    <row r="334">
+      <c r="A334" t="inlineStr">
+        <is>
+          <t>R333</t>
+        </is>
+      </c>
+      <c r="B334" t="inlineStr">
+        <is>
+          <t>pies</t>
+        </is>
+      </c>
+      <c r="C334" t="inlineStr">
+        <is>
+          <t>German Longhaired Pointer</t>
+        </is>
+      </c>
+      <c r="F334" t="n">
+        <v>1</v>
+      </c>
+      <c r="G334" t="n">
+        <v>0</v>
+      </c>
+      <c r="H334" t="n">
+        <v>0</v>
+      </c>
+      <c r="I334" t="inlineStr">
+        <is>
+          <t>German pointer (1)</t>
+        </is>
+      </c>
+      <c r="J334" t="inlineStr">
+        <is>
+          <t>Wyżeł niemiecki długowłosy</t>
+        </is>
+      </c>
+      <c r="L334" t="inlineStr">
+        <is>
+          <t>szkic (Claude, 27.10.2026)</t>
+        </is>
+      </c>
+      <c r="M334" t="inlineStr">
+        <is>
+          <t>Deutsch Langhaar</t>
+        </is>
+      </c>
+      <c r="N334" t="inlineStr">
+        <is>
+          <t>szkic (Claude, 27.10.2026)</t>
+        </is>
+      </c>
+      <c r="O334" t="inlineStr">
+        <is>
+          <t>Chien d'arrêt allemand à poil long</t>
+        </is>
+      </c>
+      <c r="P334" t="inlineStr">
+        <is>
+          <t>szkic (Claude, 27.10.2026)</t>
+        </is>
+      </c>
+      <c r="Q334" t="inlineStr">
+        <is>
+          <t>Perro de muestra alemán de pelo largo</t>
+        </is>
+      </c>
+      <c r="R334" t="inlineStr">
+        <is>
+          <t>szkic (Claude, 27.10.2026)</t>
+        </is>
+      </c>
+      <c r="S334" t="inlineStr">
+        <is>
+          <t>Duitse langhaar</t>
+        </is>
+      </c>
+      <c r="T334" t="inlineStr">
+        <is>
+          <t>szkic (Claude, 27.10.2026)</t>
+        </is>
+      </c>
+      <c r="U334" t="inlineStr">
+        <is>
+          <t>Bracco tedesco a pelo lungo</t>
+        </is>
+      </c>
+      <c r="V334" t="inlineStr">
+        <is>
+          <t>szkic (Claude, 27.10.2026)</t>
+        </is>
+      </c>
+      <c r="W334" t="inlineStr">
+        <is>
+          <t>Braco alemão de pelo comprido</t>
+        </is>
+      </c>
+      <c r="X334" t="inlineStr">
+        <is>
+          <t>szkic (Claude, 27.10.2026)</t>
+        </is>
+      </c>
+      <c r="Y334" t="inlineStr">
+        <is>
+          <t>Deutsch Langhaar</t>
+        </is>
+      </c>
+      <c r="Z334" t="inlineStr">
+        <is>
+          <t>szkic (Claude, 27.10.2026)</t>
+        </is>
+      </c>
+      <c r="AB334" t="inlineStr">
+        <is>
+          <t>Dodana 27.10.2026 na polecenie właścicielki (rasa wskazana dla oferty 664742594). Tłumaczenia to szkice Claude'a (wzorzec jak German Wirehaired Pointer), do sprawdzenia.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Rasy.xlsx: zatwierdzone tłumaczenia R332/R333; Wirehaired Vizsla (PL nazwa, bez synonimu); stan prac
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_019xek4mwGKLwNoADM59d9Qh
</commit_message>
<xml_diff>
--- a/data/Rasy.xlsx
+++ b/data/Rasy.xlsx
@@ -37424,7 +37424,7 @@
       </c>
       <c r="L333" t="inlineStr">
         <is>
-          <t>szkic (Claude, 27.10.2026)</t>
+          <t>zatwierdzone (właścicielka)</t>
         </is>
       </c>
       <c r="M333" t="inlineStr">
@@ -37434,7 +37434,7 @@
       </c>
       <c r="N333" t="inlineStr">
         <is>
-          <t>szkic (Claude, 27.10.2026)</t>
+          <t>zatwierdzone (właścicielka)</t>
         </is>
       </c>
       <c r="O333" t="inlineStr">
@@ -37444,7 +37444,7 @@
       </c>
       <c r="P333" t="inlineStr">
         <is>
-          <t>szkic (Claude, 27.10.2026)</t>
+          <t>zatwierdzone (właścicielka)</t>
         </is>
       </c>
       <c r="Q333" t="inlineStr">
@@ -37454,7 +37454,7 @@
       </c>
       <c r="R333" t="inlineStr">
         <is>
-          <t>szkic (Claude, 27.10.2026)</t>
+          <t>zatwierdzone (właścicielka)</t>
         </is>
       </c>
       <c r="S333" t="inlineStr">
@@ -37464,7 +37464,7 @@
       </c>
       <c r="T333" t="inlineStr">
         <is>
-          <t>szkic (Claude, 27.10.2026)</t>
+          <t>zatwierdzone (właścicielka)</t>
         </is>
       </c>
       <c r="U333" t="inlineStr">
@@ -37474,7 +37474,7 @@
       </c>
       <c r="V333" t="inlineStr">
         <is>
-          <t>szkic (Claude, 27.10.2026)</t>
+          <t>zatwierdzone (właścicielka)</t>
         </is>
       </c>
       <c r="W333" t="inlineStr">
@@ -37484,7 +37484,7 @@
       </c>
       <c r="X333" t="inlineStr">
         <is>
-          <t>szkic (Claude, 27.10.2026)</t>
+          <t>zatwierdzone (właścicielka)</t>
         </is>
       </c>
       <c r="Y333" t="inlineStr">
@@ -37494,12 +37494,12 @@
       </c>
       <c r="Z333" t="inlineStr">
         <is>
-          <t>szkic (Claude, 27.10.2026)</t>
+          <t>zatwierdzone (właścicielka)</t>
         </is>
       </c>
       <c r="AB333" t="inlineStr">
         <is>
-          <t>Dodana 27.10.2026 na polecenie właścicielki (rasa wskazana dla oferty 664703588). Tłumaczenia to szkice Claude'a do sprawdzenia.</t>
+          <t>Dodana 27.10.2026 na polecenie właścicielki (rasa wskazana dla oferty 664703588). Tłumaczenia to szkice Claude'a do sprawdzenia. Tłumaczenia zatwierdzone przez właścicielkę 27.10.2026 (bez weryfikacji natywnej).</t>
         </is>
       </c>
     </row>
@@ -37540,7 +37540,7 @@
       </c>
       <c r="L334" t="inlineStr">
         <is>
-          <t>szkic (Claude, 27.10.2026)</t>
+          <t>zatwierdzone (właścicielka)</t>
         </is>
       </c>
       <c r="M334" t="inlineStr">
@@ -37550,7 +37550,7 @@
       </c>
       <c r="N334" t="inlineStr">
         <is>
-          <t>szkic (Claude, 27.10.2026)</t>
+          <t>zatwierdzone (właścicielka)</t>
         </is>
       </c>
       <c r="O334" t="inlineStr">
@@ -37560,7 +37560,7 @@
       </c>
       <c r="P334" t="inlineStr">
         <is>
-          <t>szkic (Claude, 27.10.2026)</t>
+          <t>zatwierdzone (właścicielka)</t>
         </is>
       </c>
       <c r="Q334" t="inlineStr">
@@ -37570,7 +37570,7 @@
       </c>
       <c r="R334" t="inlineStr">
         <is>
-          <t>szkic (Claude, 27.10.2026)</t>
+          <t>zatwierdzone (właścicielka)</t>
         </is>
       </c>
       <c r="S334" t="inlineStr">
@@ -37580,7 +37580,7 @@
       </c>
       <c r="T334" t="inlineStr">
         <is>
-          <t>szkic (Claude, 27.10.2026)</t>
+          <t>zatwierdzone (właścicielka)</t>
         </is>
       </c>
       <c r="U334" t="inlineStr">
@@ -37590,7 +37590,7 @@
       </c>
       <c r="V334" t="inlineStr">
         <is>
-          <t>szkic (Claude, 27.10.2026)</t>
+          <t>zatwierdzone (właścicielka)</t>
         </is>
       </c>
       <c r="W334" t="inlineStr">
@@ -37600,7 +37600,7 @@
       </c>
       <c r="X334" t="inlineStr">
         <is>
-          <t>szkic (Claude, 27.10.2026)</t>
+          <t>zatwierdzone (właścicielka)</t>
         </is>
       </c>
       <c r="Y334" t="inlineStr">
@@ -37610,12 +37610,12 @@
       </c>
       <c r="Z334" t="inlineStr">
         <is>
-          <t>szkic (Claude, 27.10.2026)</t>
+          <t>zatwierdzone (właścicielka)</t>
         </is>
       </c>
       <c r="AB334" t="inlineStr">
         <is>
-          <t>Dodana 27.10.2026 na polecenie właścicielki (rasa wskazana dla oferty 664742594). Tłumaczenia to szkice Claude'a (wzorzec jak German Wirehaired Pointer), do sprawdzenia.</t>
+          <t>Dodana 27.10.2026 na polecenie właścicielki (rasa wskazana dla oferty 664742594). Tłumaczenia to szkice Claude'a (wzorzec jak German Wirehaired Pointer), do sprawdzenia. Tłumaczenia zatwierdzone przez właścicielkę 27.10.2026 (bez weryfikacji natywnej).</t>
         </is>
       </c>
     </row>

</xml_diff>